<commit_message>
Update attendance data 2026-07-02
</commit_message>
<xml_diff>
--- a/Caleb_2026.xlsx
+++ b/Caleb_2026.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="26">
   <si>
     <t>月份</t>
   </si>
@@ -1180,6 +1180,12 @@
       <c r="L4" t="s">
         <v>9</v>
       </c>
+      <c r="M4" t="s">
+        <v>9</v>
+      </c>
+      <c r="N4" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -1206,6 +1212,12 @@
       <c r="L5" t="s">
         <v>9</v>
       </c>
+      <c r="M5" t="s">
+        <v>9</v>
+      </c>
+      <c r="N5" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -1229,6 +1241,12 @@
       <c r="L6" t="s">
         <v>9</v>
       </c>
+      <c r="M6" t="s">
+        <v>9</v>
+      </c>
+      <c r="N6" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -1253,6 +1271,12 @@
         <v>9</v>
       </c>
       <c r="L7" t="s">
+        <v>9</v>
+      </c>
+      <c r="M7" t="s">
+        <v>9</v>
+      </c>
+      <c r="N7" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>